<commit_message>
feat(perf & ui): system-wide speedup, skeleton loaders, fallbacks, and DSA optimizations
</commit_message>
<xml_diff>
--- a/docs/Tower -A.xlsx
+++ b/docs/Tower -A.xlsx
@@ -3,17 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_37DC09B0030E803D57F91A838FC6C4200DBE5D40" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CDE14F13-CF5C-49FD-80F2-0F947E83FCE0}"/>
+  <xr:revisionPtr revIDLastSave="232" documentId="11_37DC09B0030E803D57F91A838FC6C4200DBE5D40" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E73EF76F-09DC-4630-B7BF-0198089E7868}"/>
   <bookViews>
-    <workbookView xWindow="1770" yWindow="1770" windowWidth="21600" windowHeight="11295" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="1770" yWindow="1770" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="For Bank" sheetId="1" r:id="rId1"/>
     <sheet name="Master File" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="8" r:id="rId3"/>
+    <sheet name="Sheet1" sheetId="9" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="8" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
     <externalReference r:id="rId5"/>
     <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
@@ -190,6 +190,7 @@
     <externalReference r:id="rId178"/>
     <externalReference r:id="rId179"/>
     <externalReference r:id="rId180"/>
+    <externalReference r:id="rId181"/>
   </externalReferences>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'For Bank'!$A$7:$O$139</definedName>
@@ -417,6 +418,90 @@
     <author>Author</author>
   </authors>
   <commentList>
+    <comment ref="B19" authorId="0" shapeId="0" xr:uid="{23AF7DE0-DF2B-4EFF-9801-F924D1451D75}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Flat No. A - 503
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B20" authorId="0" shapeId="0" xr:uid="{CF32B9C5-1F10-42F9-814E-A12E81F13E55}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Flat No. A - 503
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B23" authorId="0" shapeId="0" xr:uid="{DDAB8C19-BEEB-4D50-A1A9-1CA3BA351E38}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Flat No. A - 704
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B27" authorId="0" shapeId="0" xr:uid="{6DD38F8E-EC9F-4708-AC5B-6F29E0729899}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">MOU in the Flat no. 610
+</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C38" authorId="0" shapeId="0" xr:uid="{DC1BE483-E7DC-492F-989D-71FCA609F8CB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Cancelled</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Author</author>
+  </authors>
+  <commentList>
     <comment ref="B17" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0200-000001000000}">
       <text>
         <r>
@@ -467,7 +552,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2214" uniqueCount="980">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2426" uniqueCount="980">
   <si>
     <t>Particulars</t>
   </si>
@@ -4971,6 +5056,15 @@
     </xf>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="2" fillId="6" borderId="19" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="14" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -5001,15 +5095,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -19817,6 +19902,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -20109,6 +20198,18 @@
   <wetp:taskpane dockstate="right" visibility="0" width="350" row="1">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="460" row="1">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+  </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="3">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+  </wetp:taskpane>
+  <wetp:taskpane dockstate="right" visibility="0" width="350" row="4">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+  </wetp:taskpane>
 </wetp:taskpanes>
 </file>
 
@@ -20123,6 +20224,99 @@
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension2.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{6A0624C2-7566-4385-980C-72BDFF56F594}">
+  <we:reference id="wa200005669" version="2.0.0.0" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005669" version="2.0.0.0" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension3.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{884B373A-21C7-4C55-9DA5-35B9DD894947}">
+  <we:reference id="wa200005502" version="1.0.0.13" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005502" version="1.0.0.13" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="docId" value="&quot;9NWU3oqYDcrS4LgpDERLN&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_GPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CREATE_PROMPT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_LIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HLIST</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CLASSIFY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TRANSLATE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EXTRACT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TAG</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_CONVERT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FORMAT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SUMMARIZE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_TABLE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_FILL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_SPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_HSPLIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_EDIT</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_MATCH</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_VISION</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GPT_WEB</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension4.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{9346AF46-CEAC-4B75-91C6-B6E40D7D9218}">
+  <we:reference id="wa200005281" version="1.0.0.0" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200005281" version="1.0.0.0" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_NUM_AI</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_NUM_WRITE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_NUM_INFER</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
+</we:webextension>
+</file>
+
+<file path=xl/webextensions/webextension5.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{46DC43AE-4EC2-4DA7-9080-D165B3E110FD}">
+  <we:reference id="wa200000556" version="1.1.0.0" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200000556" version="1.1.0.0" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="documentId" value="&quot;05c664f0-30d8-4357-ad08-fc11d78904e9&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+  <we:extLst>
+    <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
+      <we:customFunctionIdList>
+        <we:customFunctionIds>_xldudf_JIRA_JQL</we:customFunctionIds>
+      </we:customFunctionIdList>
+    </a:ext>
+  </we:extLst>
 </we:webextension>
 </file>
 
@@ -20151,55 +20345,55 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A1" s="520" t="s">
+      <c r="A1" s="508" t="s">
         <v>711</v>
       </c>
-      <c r="B1" s="520"/>
-      <c r="C1" s="520"/>
-      <c r="D1" s="520"/>
-      <c r="E1" s="520"/>
-      <c r="F1" s="520"/>
-      <c r="G1" s="520"/>
-      <c r="H1" s="520"/>
-      <c r="I1" s="520"/>
-      <c r="J1" s="520"/>
-      <c r="K1" s="520"/>
-      <c r="L1" s="520"/>
-      <c r="M1" s="520"/>
+      <c r="B1" s="508"/>
+      <c r="C1" s="508"/>
+      <c r="D1" s="508"/>
+      <c r="E1" s="508"/>
+      <c r="F1" s="508"/>
+      <c r="G1" s="508"/>
+      <c r="H1" s="508"/>
+      <c r="I1" s="508"/>
+      <c r="J1" s="508"/>
+      <c r="K1" s="508"/>
+      <c r="L1" s="508"/>
+      <c r="M1" s="508"/>
     </row>
     <row r="2" spans="1:15" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A2" s="520" t="s">
+      <c r="A2" s="508" t="s">
         <v>713</v>
       </c>
-      <c r="B2" s="520"/>
-      <c r="C2" s="520"/>
-      <c r="D2" s="520"/>
-      <c r="E2" s="520"/>
-      <c r="F2" s="520"/>
-      <c r="G2" s="520"/>
-      <c r="H2" s="520"/>
-      <c r="I2" s="520"/>
-      <c r="J2" s="520"/>
-      <c r="K2" s="520"/>
-      <c r="L2" s="520"/>
-      <c r="M2" s="520"/>
+      <c r="B2" s="508"/>
+      <c r="C2" s="508"/>
+      <c r="D2" s="508"/>
+      <c r="E2" s="508"/>
+      <c r="F2" s="508"/>
+      <c r="G2" s="508"/>
+      <c r="H2" s="508"/>
+      <c r="I2" s="508"/>
+      <c r="J2" s="508"/>
+      <c r="K2" s="508"/>
+      <c r="L2" s="508"/>
+      <c r="M2" s="508"/>
     </row>
     <row r="3" spans="1:15" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="520" t="s">
+      <c r="A3" s="508" t="s">
         <v>712</v>
       </c>
-      <c r="B3" s="520"/>
-      <c r="C3" s="520"/>
-      <c r="D3" s="520"/>
-      <c r="E3" s="520"/>
-      <c r="F3" s="520"/>
-      <c r="G3" s="520"/>
-      <c r="H3" s="520"/>
-      <c r="I3" s="520"/>
-      <c r="J3" s="520"/>
-      <c r="K3" s="520"/>
-      <c r="L3" s="520"/>
-      <c r="M3" s="520"/>
+      <c r="B3" s="508"/>
+      <c r="C3" s="508"/>
+      <c r="D3" s="508"/>
+      <c r="E3" s="508"/>
+      <c r="F3" s="508"/>
+      <c r="G3" s="508"/>
+      <c r="H3" s="508"/>
+      <c r="I3" s="508"/>
+      <c r="J3" s="508"/>
+      <c r="K3" s="508"/>
+      <c r="L3" s="508"/>
+      <c r="M3" s="508"/>
     </row>
     <row r="4" spans="1:15" ht="32.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="58"/>
@@ -20217,18 +20411,18 @@
       <c r="M4" s="58"/>
     </row>
     <row r="5" spans="1:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="509" t="s">
+      <c r="A5" s="512" t="s">
         <v>0</v>
       </c>
       <c r="B5" s="521"/>
       <c r="C5" s="522"/>
-      <c r="E5" s="512" t="s">
+      <c r="E5" s="515" t="s">
         <v>1</v>
       </c>
-      <c r="F5" s="513"/>
-      <c r="G5" s="513"/>
-      <c r="H5" s="514"/>
-      <c r="J5" s="509" t="s">
+      <c r="F5" s="516"/>
+      <c r="G5" s="516"/>
+      <c r="H5" s="517"/>
+      <c r="J5" s="512" t="s">
         <v>2</v>
       </c>
       <c r="K5" s="521"/>
@@ -25297,9 +25491,9 @@
     <col min="3" max="3" width="22.85546875" style="3" customWidth="1"/>
     <col min="4" max="4" width="15.85546875" style="3" customWidth="1"/>
     <col min="5" max="5" width="10.5703125" style="45" customWidth="1"/>
-    <col min="6" max="6" width="23" style="45" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="1.42578125" style="45" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="2.28515625" style="45" hidden="1" customWidth="1"/>
+    <col min="6" max="6" width="23.5703125" style="45" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.85546875" style="45" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="45" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15" style="62" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.42578125" style="318" customWidth="1"/>
     <col min="11" max="11" width="14.140625" style="318" customWidth="1"/>
@@ -25307,8 +25501,8 @@
     <col min="13" max="13" width="6.85546875" style="1" customWidth="1"/>
     <col min="14" max="14" width="7.7109375" style="74" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="9.28515625" style="74" customWidth="1"/>
-    <col min="16" max="16" width="12.7109375" style="74" customWidth="1"/>
-    <col min="17" max="17" width="5" style="2" hidden="1" customWidth="1"/>
+    <col min="16" max="16" width="14.7109375" style="74" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.42578125" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="14.85546875" style="2" bestFit="1" customWidth="1"/>
     <col min="19" max="19" width="13.5703125" style="2" customWidth="1"/>
     <col min="20" max="20" width="15.140625" style="2" customWidth="1"/>
@@ -25319,75 +25513,75 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A1" s="520"/>
-      <c r="B1" s="520"/>
-      <c r="C1" s="520"/>
-      <c r="D1" s="520"/>
-      <c r="E1" s="520"/>
-      <c r="F1" s="520"/>
-      <c r="G1" s="520"/>
-      <c r="H1" s="520"/>
-      <c r="I1" s="520"/>
-      <c r="J1" s="520"/>
-      <c r="K1" s="520"/>
-      <c r="L1" s="520"/>
-      <c r="M1" s="518"/>
-      <c r="N1" s="519"/>
-      <c r="O1" s="519"/>
-      <c r="P1" s="519"/>
-      <c r="Q1" s="518"/>
-      <c r="R1" s="518"/>
-      <c r="S1" s="518"/>
-      <c r="T1" s="518"/>
-      <c r="U1" s="518"/>
+      <c r="A1" s="508"/>
+      <c r="B1" s="508"/>
+      <c r="C1" s="508"/>
+      <c r="D1" s="508"/>
+      <c r="E1" s="508"/>
+      <c r="F1" s="508"/>
+      <c r="G1" s="508"/>
+      <c r="H1" s="508"/>
+      <c r="I1" s="508"/>
+      <c r="J1" s="508"/>
+      <c r="K1" s="508"/>
+      <c r="L1" s="508"/>
+      <c r="M1" s="506"/>
+      <c r="N1" s="507"/>
+      <c r="O1" s="507"/>
+      <c r="P1" s="507"/>
+      <c r="Q1" s="506"/>
+      <c r="R1" s="506"/>
+      <c r="S1" s="506"/>
+      <c r="T1" s="506"/>
+      <c r="U1" s="506"/>
     </row>
     <row r="2" spans="1:22" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A2" s="520" t="s">
+      <c r="A2" s="508" t="s">
         <v>713</v>
       </c>
-      <c r="B2" s="520"/>
-      <c r="C2" s="520"/>
-      <c r="D2" s="520"/>
-      <c r="E2" s="520"/>
-      <c r="F2" s="520"/>
-      <c r="G2" s="520"/>
-      <c r="H2" s="520"/>
-      <c r="I2" s="520"/>
-      <c r="J2" s="520"/>
-      <c r="K2" s="520"/>
-      <c r="L2" s="520"/>
-      <c r="M2" s="518"/>
-      <c r="N2" s="519"/>
-      <c r="O2" s="519"/>
-      <c r="P2" s="519"/>
-      <c r="Q2" s="518"/>
-      <c r="R2" s="518"/>
-      <c r="S2" s="518"/>
-      <c r="T2" s="518"/>
-      <c r="U2" s="518"/>
+      <c r="B2" s="508"/>
+      <c r="C2" s="508"/>
+      <c r="D2" s="508"/>
+      <c r="E2" s="508"/>
+      <c r="F2" s="508"/>
+      <c r="G2" s="508"/>
+      <c r="H2" s="508"/>
+      <c r="I2" s="508"/>
+      <c r="J2" s="508"/>
+      <c r="K2" s="508"/>
+      <c r="L2" s="508"/>
+      <c r="M2" s="506"/>
+      <c r="N2" s="507"/>
+      <c r="O2" s="507"/>
+      <c r="P2" s="507"/>
+      <c r="Q2" s="506"/>
+      <c r="R2" s="506"/>
+      <c r="S2" s="506"/>
+      <c r="T2" s="506"/>
+      <c r="U2" s="506"/>
     </row>
     <row r="3" spans="1:22" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A3" s="520"/>
-      <c r="B3" s="520"/>
-      <c r="C3" s="520"/>
-      <c r="D3" s="520"/>
-      <c r="E3" s="520"/>
-      <c r="F3" s="520"/>
-      <c r="G3" s="520"/>
-      <c r="H3" s="520"/>
-      <c r="I3" s="520"/>
-      <c r="J3" s="520"/>
-      <c r="K3" s="520"/>
-      <c r="L3" s="520"/>
-      <c r="M3" s="518"/>
-      <c r="N3" s="519"/>
-      <c r="O3" s="519"/>
-      <c r="P3" s="519"/>
-      <c r="Q3" s="518"/>
-      <c r="R3" s="518"/>
-      <c r="S3" s="518"/>
-      <c r="T3" s="518"/>
-      <c r="U3" s="518"/>
+      <c r="A3" s="508"/>
+      <c r="B3" s="508"/>
+      <c r="C3" s="508"/>
+      <c r="D3" s="508"/>
+      <c r="E3" s="508"/>
+      <c r="F3" s="508"/>
+      <c r="G3" s="508"/>
+      <c r="H3" s="508"/>
+      <c r="I3" s="508"/>
+      <c r="J3" s="508"/>
+      <c r="K3" s="508"/>
+      <c r="L3" s="508"/>
+      <c r="M3" s="506"/>
+      <c r="N3" s="507"/>
+      <c r="O3" s="507"/>
+      <c r="P3" s="507"/>
+      <c r="Q3" s="506"/>
+      <c r="R3" s="506"/>
+      <c r="S3" s="506"/>
+      <c r="T3" s="506"/>
+      <c r="U3" s="506"/>
     </row>
     <row r="4" spans="1:22" ht="32.25" thickBot="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="58"/>
@@ -25400,36 +25594,36 @@
       <c r="H4" s="58"/>
     </row>
     <row r="5" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="509" t="s">
-        <v>0</v>
-      </c>
-      <c r="B5" s="510"/>
-      <c r="C5" s="511"/>
+      <c r="A5" s="512" t="s">
+        <v>0</v>
+      </c>
+      <c r="B5" s="513"/>
+      <c r="C5" s="514"/>
       <c r="D5" s="317"/>
-      <c r="E5" s="512" t="s">
+      <c r="E5" s="515" t="s">
         <v>562</v>
       </c>
-      <c r="F5" s="513"/>
-      <c r="G5" s="513"/>
-      <c r="H5" s="514"/>
-      <c r="I5" s="506" t="s">
+      <c r="F5" s="516"/>
+      <c r="G5" s="516"/>
+      <c r="H5" s="517"/>
+      <c r="I5" s="509" t="s">
         <v>563</v>
       </c>
-      <c r="J5" s="507"/>
-      <c r="K5" s="508"/>
+      <c r="J5" s="510"/>
+      <c r="K5" s="511"/>
       <c r="L5" s="354" t="s">
         <v>564</v>
       </c>
-      <c r="M5" s="515"/>
-      <c r="N5" s="516"/>
-      <c r="O5" s="516"/>
-      <c r="P5" s="517"/>
-      <c r="R5" s="506" t="s">
+      <c r="M5" s="518"/>
+      <c r="N5" s="519"/>
+      <c r="O5" s="519"/>
+      <c r="P5" s="520"/>
+      <c r="R5" s="509" t="s">
         <v>565</v>
       </c>
-      <c r="S5" s="507"/>
-      <c r="T5" s="507"/>
-      <c r="U5" s="508"/>
+      <c r="S5" s="510"/>
+      <c r="T5" s="510"/>
+      <c r="U5" s="511"/>
     </row>
     <row r="6" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
@@ -39270,17 +39464,17 @@
   </sheetData>
   <autoFilter ref="A7:U220" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <mergeCells count="11">
+    <mergeCell ref="R5:U5"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="M5:P5"/>
     <mergeCell ref="M1:U1"/>
     <mergeCell ref="M2:U2"/>
     <mergeCell ref="M3:U3"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A2:L2"/>
     <mergeCell ref="A3:L3"/>
-    <mergeCell ref="R5:U5"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="M5:P5"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="41" orientation="landscape" r:id="rId1"/>
@@ -39289,6 +39483,3290 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC38D4E8-CB90-4D88-8854-DF9153700544}">
+  <dimension ref="A1:V52"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="12" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="20" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="208">
+        <v>19</v>
+      </c>
+      <c r="B1" s="209" t="s">
+        <v>48</v>
+      </c>
+      <c r="C1" s="86" t="s">
+        <v>606</v>
+      </c>
+      <c r="D1" s="368" t="s">
+        <v>929</v>
+      </c>
+      <c r="E1" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G1" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H1" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I1" s="212">
+        <v>41711</v>
+      </c>
+      <c r="J1" s="326">
+        <v>41739</v>
+      </c>
+      <c r="K1" s="345">
+        <v>44752</v>
+      </c>
+      <c r="L1" s="359">
+        <v>45361</v>
+      </c>
+      <c r="M1" s="213">
+        <v>100</v>
+      </c>
+      <c r="N1" s="214">
+        <v>0</v>
+      </c>
+      <c r="O1" s="214">
+        <v>100</v>
+      </c>
+      <c r="P1" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q1" s="80"/>
+      <c r="R1" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S1" s="216">
+        <v>0</v>
+      </c>
+      <c r="T1" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U1" s="215"/>
+    </row>
+    <row r="2" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A2" s="208">
+        <v>29</v>
+      </c>
+      <c r="B2" s="209" t="s">
+        <v>52</v>
+      </c>
+      <c r="C2" s="86" t="s">
+        <v>607</v>
+      </c>
+      <c r="D2" s="368" t="s">
+        <v>929</v>
+      </c>
+      <c r="E2" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G2" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H2" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I2" s="212">
+        <v>41787</v>
+      </c>
+      <c r="J2" s="326">
+        <v>41800</v>
+      </c>
+      <c r="K2" s="345">
+        <v>44814</v>
+      </c>
+      <c r="L2" s="359">
+        <v>45422</v>
+      </c>
+      <c r="M2" s="213">
+        <v>100</v>
+      </c>
+      <c r="N2" s="214">
+        <v>0</v>
+      </c>
+      <c r="O2" s="214">
+        <v>100</v>
+      </c>
+      <c r="P2" s="214">
+        <v>0</v>
+      </c>
+      <c r="R2" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S2" s="216">
+        <v>0</v>
+      </c>
+      <c r="T2" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U2" s="215">
+        <v>0</v>
+      </c>
+      <c r="V2" s="80" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A3" s="155">
+        <v>31</v>
+      </c>
+      <c r="B3" s="96" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="94" t="s">
+        <v>608</v>
+      </c>
+      <c r="D3" s="371" t="s">
+        <v>929</v>
+      </c>
+      <c r="E3" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G3" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H3" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I3" s="89">
+        <v>41744</v>
+      </c>
+      <c r="J3" s="328">
+        <v>41769</v>
+      </c>
+      <c r="K3" s="347">
+        <v>44783</v>
+      </c>
+      <c r="L3" s="361">
+        <v>45392</v>
+      </c>
+      <c r="M3" s="90">
+        <v>100</v>
+      </c>
+      <c r="N3" s="91">
+        <v>0</v>
+      </c>
+      <c r="O3" s="91">
+        <v>100</v>
+      </c>
+      <c r="P3" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="80"/>
+      <c r="R3" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S3" s="93">
+        <v>0</v>
+      </c>
+      <c r="T3" s="93">
+        <v>1568000</v>
+      </c>
+      <c r="U3" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A4" s="155">
+        <v>33</v>
+      </c>
+      <c r="B4" s="96" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="99" t="s">
+        <v>610</v>
+      </c>
+      <c r="D4" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E4" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G4" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H4" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I4" s="89">
+        <v>41657</v>
+      </c>
+      <c r="J4" s="328">
+        <v>41680</v>
+      </c>
+      <c r="K4" s="347">
+        <v>44691</v>
+      </c>
+      <c r="L4" s="361">
+        <v>45301</v>
+      </c>
+      <c r="M4" s="90">
+        <v>100</v>
+      </c>
+      <c r="N4" s="91">
+        <v>0</v>
+      </c>
+      <c r="O4" s="91">
+        <v>100</v>
+      </c>
+      <c r="P4" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S4" s="93">
+        <v>0</v>
+      </c>
+      <c r="T4" s="93">
+        <v>1600000</v>
+      </c>
+      <c r="U4" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" s="78" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="155">
+        <v>34</v>
+      </c>
+      <c r="B5" s="96" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="99" t="s">
+        <v>710</v>
+      </c>
+      <c r="D5" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E5" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" s="88">
+        <v>22000</v>
+      </c>
+      <c r="G5" s="88">
+        <v>2200</v>
+      </c>
+      <c r="H5" s="88">
+        <v>19800</v>
+      </c>
+      <c r="I5" s="89">
+        <v>42128</v>
+      </c>
+      <c r="J5" s="328">
+        <v>42165</v>
+      </c>
+      <c r="K5" s="347">
+        <v>45179</v>
+      </c>
+      <c r="L5" s="361">
+        <v>45787</v>
+      </c>
+      <c r="M5" s="90">
+        <v>100</v>
+      </c>
+      <c r="N5" s="91">
+        <v>7</v>
+      </c>
+      <c r="O5" s="91">
+        <v>93</v>
+      </c>
+      <c r="P5" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="80"/>
+      <c r="R5" s="92">
+        <v>2151000</v>
+      </c>
+      <c r="S5" s="93">
+        <v>105000</v>
+      </c>
+      <c r="T5" s="93">
+        <v>2046000</v>
+      </c>
+      <c r="U5" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A6" s="239">
+        <v>39</v>
+      </c>
+      <c r="B6" s="159" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="240" t="s">
+        <v>614</v>
+      </c>
+      <c r="D6" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E6" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G6" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H6" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I6" s="242">
+        <v>41787</v>
+      </c>
+      <c r="J6" s="330">
+        <v>41800</v>
+      </c>
+      <c r="K6" s="349">
+        <v>44814</v>
+      </c>
+      <c r="L6" s="349">
+        <v>45422</v>
+      </c>
+      <c r="M6" s="239">
+        <v>100</v>
+      </c>
+      <c r="N6" s="243">
+        <v>0</v>
+      </c>
+      <c r="O6" s="243">
+        <v>100</v>
+      </c>
+      <c r="P6" s="243">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="80"/>
+      <c r="R6" s="241">
+        <v>1600000</v>
+      </c>
+      <c r="S6" s="241">
+        <v>0</v>
+      </c>
+      <c r="T6" s="241">
+        <v>1568000</v>
+      </c>
+      <c r="U6" s="241">
+        <v>32000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="208">
+        <v>41</v>
+      </c>
+      <c r="B7" s="226" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" s="99" t="s">
+        <v>616</v>
+      </c>
+      <c r="D7" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E7" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F7" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G7" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H7" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I7" s="212">
+        <v>41891</v>
+      </c>
+      <c r="J7" s="326">
+        <v>41922</v>
+      </c>
+      <c r="K7" s="345">
+        <v>44936</v>
+      </c>
+      <c r="L7" s="359">
+        <v>45545</v>
+      </c>
+      <c r="M7" s="213">
+        <v>100</v>
+      </c>
+      <c r="N7" s="214">
+        <v>0</v>
+      </c>
+      <c r="O7" s="214">
+        <v>100</v>
+      </c>
+      <c r="P7" s="214">
+        <v>0</v>
+      </c>
+      <c r="R7" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S7" s="216">
+        <v>0</v>
+      </c>
+      <c r="T7" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U7" s="215">
+        <v>0</v>
+      </c>
+      <c r="V7" s="80" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A8" s="239">
+        <v>42</v>
+      </c>
+      <c r="B8" s="159" t="s">
+        <v>106</v>
+      </c>
+      <c r="C8" s="240" t="s">
+        <v>617</v>
+      </c>
+      <c r="D8" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E8" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G8" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H8" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I8" s="242">
+        <v>41827</v>
+      </c>
+      <c r="J8" s="330">
+        <v>41907</v>
+      </c>
+      <c r="K8" s="349">
+        <v>44920</v>
+      </c>
+      <c r="L8" s="349">
+        <v>45529</v>
+      </c>
+      <c r="M8" s="239">
+        <v>100</v>
+      </c>
+      <c r="N8" s="243">
+        <v>0</v>
+      </c>
+      <c r="O8" s="243">
+        <v>100</v>
+      </c>
+      <c r="P8" s="243">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="80"/>
+      <c r="R8" s="241">
+        <v>1600000</v>
+      </c>
+      <c r="S8" s="241">
+        <v>0</v>
+      </c>
+      <c r="T8" s="241">
+        <v>1584000</v>
+      </c>
+      <c r="U8" s="241">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A9" s="239">
+        <v>44</v>
+      </c>
+      <c r="B9" s="159" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="240" t="s">
+        <v>618</v>
+      </c>
+      <c r="D9" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E9" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F9" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G9" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H9" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I9" s="242">
+        <v>41795</v>
+      </c>
+      <c r="J9" s="330">
+        <v>41784</v>
+      </c>
+      <c r="K9" s="349">
+        <v>44798</v>
+      </c>
+      <c r="L9" s="349">
+        <v>45407</v>
+      </c>
+      <c r="M9" s="239">
+        <v>100</v>
+      </c>
+      <c r="N9" s="246">
+        <v>44</v>
+      </c>
+      <c r="O9" s="246">
+        <v>56</v>
+      </c>
+      <c r="P9" s="246">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="80"/>
+      <c r="R9" s="245">
+        <v>1248000</v>
+      </c>
+      <c r="S9" s="245">
+        <v>352000</v>
+      </c>
+      <c r="T9" s="245">
+        <v>896000</v>
+      </c>
+      <c r="U9" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A10" s="239">
+        <v>46</v>
+      </c>
+      <c r="B10" s="160" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="244" t="s">
+        <v>619</v>
+      </c>
+      <c r="D10" s="244" t="s">
+        <v>929</v>
+      </c>
+      <c r="E10" s="245" t="s">
+        <v>30</v>
+      </c>
+      <c r="F10" s="245">
+        <v>25000</v>
+      </c>
+      <c r="G10" s="245">
+        <v>2500</v>
+      </c>
+      <c r="H10" s="245">
+        <v>22500</v>
+      </c>
+      <c r="I10" s="242">
+        <v>42916</v>
+      </c>
+      <c r="J10" s="330">
+        <v>42941</v>
+      </c>
+      <c r="K10" s="349">
+        <v>45955</v>
+      </c>
+      <c r="L10" s="349">
+        <v>46563</v>
+      </c>
+      <c r="M10" s="247">
+        <v>100</v>
+      </c>
+      <c r="N10" s="246">
+        <v>0</v>
+      </c>
+      <c r="O10" s="246">
+        <v>69</v>
+      </c>
+      <c r="P10" s="246">
+        <v>31</v>
+      </c>
+      <c r="Q10" s="80"/>
+      <c r="R10" s="245">
+        <v>2500000</v>
+      </c>
+      <c r="S10" s="245">
+        <v>0</v>
+      </c>
+      <c r="T10" s="245">
+        <v>1725000</v>
+      </c>
+      <c r="U10" s="245">
+        <v>775000</v>
+      </c>
+    </row>
+    <row r="11" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A11" s="155">
+        <v>48</v>
+      </c>
+      <c r="B11" s="96" t="s">
+        <v>737</v>
+      </c>
+      <c r="C11" s="99" t="s">
+        <v>743</v>
+      </c>
+      <c r="D11" s="373"/>
+      <c r="E11" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G11" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H11" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I11" s="89"/>
+      <c r="J11" s="328">
+        <v>41800</v>
+      </c>
+      <c r="K11" s="347">
+        <v>44814</v>
+      </c>
+      <c r="L11" s="361">
+        <v>45422</v>
+      </c>
+      <c r="M11" s="90">
+        <v>100</v>
+      </c>
+      <c r="N11" s="91">
+        <v>0</v>
+      </c>
+      <c r="O11" s="91">
+        <v>62</v>
+      </c>
+      <c r="P11" s="91">
+        <v>38</v>
+      </c>
+      <c r="Q11" s="80"/>
+      <c r="R11" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S11" s="93">
+        <v>0</v>
+      </c>
+      <c r="T11" s="93">
+        <v>992000</v>
+      </c>
+      <c r="U11" s="92">
+        <v>608000</v>
+      </c>
+      <c r="V11" s="78" t="s">
+        <v>946</v>
+      </c>
+    </row>
+    <row r="12" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A12" s="155">
+        <v>51</v>
+      </c>
+      <c r="B12" s="96" t="s">
+        <v>131</v>
+      </c>
+      <c r="C12" s="99" t="s">
+        <v>623</v>
+      </c>
+      <c r="D12" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E12" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F12" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G12" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H12" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I12" s="89">
+        <v>41842</v>
+      </c>
+      <c r="J12" s="328">
+        <v>41861</v>
+      </c>
+      <c r="K12" s="347">
+        <v>44875</v>
+      </c>
+      <c r="L12" s="361">
+        <v>45483</v>
+      </c>
+      <c r="M12" s="90">
+        <v>100</v>
+      </c>
+      <c r="N12" s="91">
+        <v>0</v>
+      </c>
+      <c r="O12" s="91">
+        <v>100</v>
+      </c>
+      <c r="P12" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="80"/>
+      <c r="R12" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S12" s="93">
+        <v>0</v>
+      </c>
+      <c r="T12" s="93">
+        <v>1600000</v>
+      </c>
+      <c r="U12" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A13" s="239">
+        <v>56</v>
+      </c>
+      <c r="B13" s="159" t="s">
+        <v>149</v>
+      </c>
+      <c r="C13" s="240" t="s">
+        <v>625</v>
+      </c>
+      <c r="D13" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E13" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F13" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G13" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H13" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I13" s="242">
+        <v>41827</v>
+      </c>
+      <c r="J13" s="330">
+        <v>41784</v>
+      </c>
+      <c r="K13" s="349">
+        <v>44798</v>
+      </c>
+      <c r="L13" s="349">
+        <v>45407</v>
+      </c>
+      <c r="M13" s="239">
+        <v>100</v>
+      </c>
+      <c r="N13" s="246">
+        <v>47</v>
+      </c>
+      <c r="O13" s="246">
+        <v>53</v>
+      </c>
+      <c r="P13" s="246">
+        <v>0</v>
+      </c>
+      <c r="R13" s="245">
+        <v>1224000</v>
+      </c>
+      <c r="S13" s="245">
+        <v>376000</v>
+      </c>
+      <c r="T13" s="245">
+        <v>848000</v>
+      </c>
+      <c r="U13" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A14" s="155">
+        <v>60</v>
+      </c>
+      <c r="B14" s="96" t="s">
+        <v>164</v>
+      </c>
+      <c r="C14" s="94" t="s">
+        <v>628</v>
+      </c>
+      <c r="D14" s="371" t="s">
+        <v>929</v>
+      </c>
+      <c r="E14" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F14" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G14" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H14" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I14" s="89">
+        <v>41891</v>
+      </c>
+      <c r="J14" s="328">
+        <v>41892</v>
+      </c>
+      <c r="K14" s="347">
+        <v>44905</v>
+      </c>
+      <c r="L14" s="361">
+        <v>45514</v>
+      </c>
+      <c r="M14" s="90">
+        <v>100</v>
+      </c>
+      <c r="N14" s="91">
+        <v>59</v>
+      </c>
+      <c r="O14" s="91">
+        <v>41</v>
+      </c>
+      <c r="P14" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="80"/>
+      <c r="R14" s="92">
+        <v>1688500</v>
+      </c>
+      <c r="S14" s="93">
+        <v>1032500</v>
+      </c>
+      <c r="T14" s="93">
+        <v>700500</v>
+      </c>
+      <c r="U14" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="239">
+        <v>62</v>
+      </c>
+      <c r="B15" s="159" t="s">
+        <v>172</v>
+      </c>
+      <c r="C15" s="240" t="s">
+        <v>630</v>
+      </c>
+      <c r="D15" s="240"/>
+      <c r="E15" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F15" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G15" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H15" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I15" s="242">
+        <v>42010</v>
+      </c>
+      <c r="J15" s="330">
+        <v>42029</v>
+      </c>
+      <c r="K15" s="349">
+        <v>45041</v>
+      </c>
+      <c r="L15" s="349">
+        <v>45651</v>
+      </c>
+      <c r="M15" s="239">
+        <v>100</v>
+      </c>
+      <c r="N15" s="243">
+        <v>0</v>
+      </c>
+      <c r="O15" s="243">
+        <v>99</v>
+      </c>
+      <c r="P15" s="243">
+        <v>99</v>
+      </c>
+      <c r="R15" s="241">
+        <v>1600000</v>
+      </c>
+      <c r="S15" s="241">
+        <v>0</v>
+      </c>
+      <c r="T15" s="241">
+        <v>1584000</v>
+      </c>
+      <c r="U15" s="241">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A16" s="239">
+        <v>64</v>
+      </c>
+      <c r="B16" s="159" t="s">
+        <v>182</v>
+      </c>
+      <c r="C16" s="240" t="s">
+        <v>632</v>
+      </c>
+      <c r="D16" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E16" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F16" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G16" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H16" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I16" s="242">
+        <v>41865</v>
+      </c>
+      <c r="J16" s="330">
+        <v>41937</v>
+      </c>
+      <c r="K16" s="349">
+        <v>44951</v>
+      </c>
+      <c r="L16" s="349">
+        <v>45560</v>
+      </c>
+      <c r="M16" s="239">
+        <v>100</v>
+      </c>
+      <c r="N16" s="246">
+        <v>57</v>
+      </c>
+      <c r="O16" s="246">
+        <v>43</v>
+      </c>
+      <c r="P16" s="246">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="80"/>
+      <c r="R16" s="245">
+        <v>1714000</v>
+      </c>
+      <c r="S16" s="245">
+        <v>1026000</v>
+      </c>
+      <c r="T16" s="245">
+        <v>688000</v>
+      </c>
+      <c r="U16" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="155">
+        <v>66</v>
+      </c>
+      <c r="B17" s="96" t="s">
+        <v>190</v>
+      </c>
+      <c r="C17" s="99" t="s">
+        <v>633</v>
+      </c>
+      <c r="D17" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E17" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F17" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G17" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H17" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I17" s="89">
+        <v>41856</v>
+      </c>
+      <c r="J17" s="328">
+        <v>41892</v>
+      </c>
+      <c r="K17" s="347">
+        <v>44905</v>
+      </c>
+      <c r="L17" s="361">
+        <v>45514</v>
+      </c>
+      <c r="M17" s="90">
+        <v>100</v>
+      </c>
+      <c r="N17" s="91">
+        <v>57</v>
+      </c>
+      <c r="O17" s="91">
+        <v>43</v>
+      </c>
+      <c r="P17" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="80"/>
+      <c r="R17" s="92">
+        <v>1714000</v>
+      </c>
+      <c r="S17" s="93">
+        <v>1026000</v>
+      </c>
+      <c r="T17" s="93">
+        <v>688000</v>
+      </c>
+      <c r="U17" s="92">
+        <v>0</v>
+      </c>
+      <c r="V17" s="2"/>
+    </row>
+    <row r="18" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A18" s="239">
+        <v>67</v>
+      </c>
+      <c r="B18" s="159" t="s">
+        <v>195</v>
+      </c>
+      <c r="C18" s="240" t="s">
+        <v>634</v>
+      </c>
+      <c r="D18" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E18" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G18" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H18" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I18" s="242">
+        <v>41883</v>
+      </c>
+      <c r="J18" s="330">
+        <v>41876</v>
+      </c>
+      <c r="K18" s="349">
+        <v>44890</v>
+      </c>
+      <c r="L18" s="349">
+        <v>45498</v>
+      </c>
+      <c r="M18" s="239">
+        <v>100</v>
+      </c>
+      <c r="N18" s="246">
+        <v>58</v>
+      </c>
+      <c r="O18" s="246">
+        <v>0</v>
+      </c>
+      <c r="P18" s="246">
+        <v>42</v>
+      </c>
+      <c r="Q18" s="80"/>
+      <c r="R18" s="245">
+        <v>1890000</v>
+      </c>
+      <c r="S18" s="245">
+        <v>1218000</v>
+      </c>
+      <c r="T18" s="245">
+        <v>0</v>
+      </c>
+      <c r="U18" s="245">
+        <v>672000</v>
+      </c>
+    </row>
+    <row r="19" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A19" s="208">
+        <v>71</v>
+      </c>
+      <c r="B19" s="209" t="s">
+        <v>211</v>
+      </c>
+      <c r="C19" s="99" t="s">
+        <v>638</v>
+      </c>
+      <c r="D19" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E19" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F19" s="505" t="s">
+        <v>979</v>
+      </c>
+      <c r="G19" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H19" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I19" s="212">
+        <v>41780</v>
+      </c>
+      <c r="J19" s="326">
+        <v>41800</v>
+      </c>
+      <c r="K19" s="345">
+        <v>44814</v>
+      </c>
+      <c r="L19" s="359">
+        <v>45422</v>
+      </c>
+      <c r="M19" s="213">
+        <v>100</v>
+      </c>
+      <c r="N19" s="214">
+        <v>0</v>
+      </c>
+      <c r="O19" s="214">
+        <v>100</v>
+      </c>
+      <c r="P19" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="80"/>
+      <c r="R19" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S19" s="216">
+        <v>0</v>
+      </c>
+      <c r="T19" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U19" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A20" s="208">
+        <v>72</v>
+      </c>
+      <c r="B20" s="226" t="s">
+        <v>214</v>
+      </c>
+      <c r="C20" s="99" t="s">
+        <v>639</v>
+      </c>
+      <c r="D20" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E20" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G20" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H20" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I20" s="212">
+        <v>41921</v>
+      </c>
+      <c r="J20" s="326">
+        <v>41953</v>
+      </c>
+      <c r="K20" s="345">
+        <v>44967</v>
+      </c>
+      <c r="L20" s="359">
+        <v>45575</v>
+      </c>
+      <c r="M20" s="213">
+        <v>100</v>
+      </c>
+      <c r="N20" s="214">
+        <v>55</v>
+      </c>
+      <c r="O20" s="214">
+        <v>45</v>
+      </c>
+      <c r="P20" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="215">
+        <v>1710000</v>
+      </c>
+      <c r="S20" s="216">
+        <v>990000</v>
+      </c>
+      <c r="T20" s="216">
+        <v>720000</v>
+      </c>
+      <c r="U20" s="215"/>
+    </row>
+    <row r="21" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A21" s="208">
+        <v>73</v>
+      </c>
+      <c r="B21" s="226" t="s">
+        <v>219</v>
+      </c>
+      <c r="C21" s="99" t="s">
+        <v>640</v>
+      </c>
+      <c r="D21" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E21" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F21" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G21" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H21" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I21" s="212">
+        <v>41711</v>
+      </c>
+      <c r="J21" s="326">
+        <v>41739</v>
+      </c>
+      <c r="K21" s="345">
+        <v>44752</v>
+      </c>
+      <c r="L21" s="359">
+        <v>45361</v>
+      </c>
+      <c r="M21" s="213">
+        <v>100</v>
+      </c>
+      <c r="N21" s="214">
+        <v>0</v>
+      </c>
+      <c r="O21" s="214">
+        <v>100</v>
+      </c>
+      <c r="P21" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="80"/>
+      <c r="R21" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S21" s="216">
+        <v>0</v>
+      </c>
+      <c r="T21" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U21" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A22" s="155">
+        <v>75</v>
+      </c>
+      <c r="B22" s="85" t="s">
+        <v>226</v>
+      </c>
+      <c r="C22" s="99" t="s">
+        <v>227</v>
+      </c>
+      <c r="D22" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E22" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="88">
+        <v>22000</v>
+      </c>
+      <c r="G22" s="88">
+        <v>2200</v>
+      </c>
+      <c r="H22" s="88">
+        <v>19800</v>
+      </c>
+      <c r="I22" s="89">
+        <v>42024</v>
+      </c>
+      <c r="J22" s="328">
+        <v>42045</v>
+      </c>
+      <c r="K22" s="347">
+        <v>45056</v>
+      </c>
+      <c r="L22" s="361">
+        <v>45667</v>
+      </c>
+      <c r="M22" s="90">
+        <v>100</v>
+      </c>
+      <c r="N22" s="91">
+        <v>0</v>
+      </c>
+      <c r="O22" s="91">
+        <v>99</v>
+      </c>
+      <c r="P22" s="91">
+        <v>1</v>
+      </c>
+      <c r="Q22" s="2"/>
+      <c r="R22" s="92">
+        <v>2200000</v>
+      </c>
+      <c r="S22" s="93">
+        <v>0</v>
+      </c>
+      <c r="T22" s="93">
+        <v>2178000</v>
+      </c>
+      <c r="U22" s="92">
+        <v>22000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:22" s="78" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A23" s="208">
+        <v>78</v>
+      </c>
+      <c r="B23" s="209" t="s">
+        <v>236</v>
+      </c>
+      <c r="C23" s="86" t="s">
+        <v>643</v>
+      </c>
+      <c r="D23" s="368" t="s">
+        <v>929</v>
+      </c>
+      <c r="E23" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F23" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G23" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H23" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I23" s="212">
+        <v>41758</v>
+      </c>
+      <c r="J23" s="326">
+        <v>41800</v>
+      </c>
+      <c r="K23" s="345">
+        <v>44814</v>
+      </c>
+      <c r="L23" s="359">
+        <v>45422</v>
+      </c>
+      <c r="M23" s="213">
+        <v>100</v>
+      </c>
+      <c r="N23" s="214">
+        <v>0</v>
+      </c>
+      <c r="O23" s="214">
+        <v>100</v>
+      </c>
+      <c r="P23" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="80"/>
+      <c r="R23" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S23" s="216">
+        <v>0</v>
+      </c>
+      <c r="T23" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U23" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="155">
+        <v>79</v>
+      </c>
+      <c r="B24" s="96" t="s">
+        <v>241</v>
+      </c>
+      <c r="C24" s="99" t="s">
+        <v>632</v>
+      </c>
+      <c r="D24" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E24" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F24" s="88">
+        <v>28500</v>
+      </c>
+      <c r="G24" s="88">
+        <v>2850</v>
+      </c>
+      <c r="H24" s="88">
+        <v>25650</v>
+      </c>
+      <c r="I24" s="89">
+        <v>43671</v>
+      </c>
+      <c r="J24" s="328">
+        <v>43656</v>
+      </c>
+      <c r="K24" s="347">
+        <v>46670</v>
+      </c>
+      <c r="L24" s="361">
+        <v>47279</v>
+      </c>
+      <c r="M24" s="90">
+        <v>100</v>
+      </c>
+      <c r="N24" s="91">
+        <v>0</v>
+      </c>
+      <c r="O24" s="91">
+        <v>56</v>
+      </c>
+      <c r="P24" s="91">
+        <v>44</v>
+      </c>
+      <c r="Q24" s="80"/>
+      <c r="R24" s="92">
+        <v>2850000</v>
+      </c>
+      <c r="S24" s="93">
+        <v>0</v>
+      </c>
+      <c r="T24" s="93">
+        <v>1596000</v>
+      </c>
+      <c r="U24" s="92">
+        <v>1254000</v>
+      </c>
+    </row>
+    <row r="25" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A25" s="155">
+        <v>83</v>
+      </c>
+      <c r="B25" s="96" t="s">
+        <v>256</v>
+      </c>
+      <c r="C25" s="99" t="s">
+        <v>647</v>
+      </c>
+      <c r="D25" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E25" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F25" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G25" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H25" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I25" s="89">
+        <v>41827</v>
+      </c>
+      <c r="J25" s="328">
+        <v>41861</v>
+      </c>
+      <c r="K25" s="347">
+        <v>44875</v>
+      </c>
+      <c r="L25" s="361">
+        <v>45483</v>
+      </c>
+      <c r="M25" s="90">
+        <v>100</v>
+      </c>
+      <c r="N25" s="91">
+        <v>58</v>
+      </c>
+      <c r="O25" s="91">
+        <v>42</v>
+      </c>
+      <c r="P25" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="80"/>
+      <c r="R25" s="92">
+        <v>1716000</v>
+      </c>
+      <c r="S25" s="93">
+        <v>1044000</v>
+      </c>
+      <c r="T25" s="93">
+        <v>672000</v>
+      </c>
+      <c r="U25" s="92">
+        <v>0</v>
+      </c>
+      <c r="V25" s="78" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="26" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A26" s="155">
+        <v>84</v>
+      </c>
+      <c r="B26" s="96" t="s">
+        <v>261</v>
+      </c>
+      <c r="C26" s="99" t="s">
+        <v>648</v>
+      </c>
+      <c r="D26" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E26" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G26" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H26" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I26" s="89">
+        <v>41851</v>
+      </c>
+      <c r="J26" s="328">
+        <v>41861</v>
+      </c>
+      <c r="K26" s="347">
+        <v>44875</v>
+      </c>
+      <c r="L26" s="361">
+        <v>45483</v>
+      </c>
+      <c r="M26" s="90">
+        <v>100</v>
+      </c>
+      <c r="N26" s="91">
+        <v>58</v>
+      </c>
+      <c r="O26" s="91">
+        <v>42</v>
+      </c>
+      <c r="P26" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="80"/>
+      <c r="R26" s="92">
+        <v>1716000</v>
+      </c>
+      <c r="S26" s="93">
+        <v>1044000</v>
+      </c>
+      <c r="T26" s="93">
+        <v>672000</v>
+      </c>
+      <c r="U26" s="92">
+        <v>0</v>
+      </c>
+      <c r="V26" s="78" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="27" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="208">
+        <v>87</v>
+      </c>
+      <c r="B27" s="226" t="s">
+        <v>280</v>
+      </c>
+      <c r="C27" s="99" t="s">
+        <v>650</v>
+      </c>
+      <c r="D27" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E27" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F27" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G27" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H27" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I27" s="212">
+        <v>41711</v>
+      </c>
+      <c r="J27" s="326">
+        <v>41769</v>
+      </c>
+      <c r="K27" s="345">
+        <v>44783</v>
+      </c>
+      <c r="L27" s="359">
+        <v>45392</v>
+      </c>
+      <c r="M27" s="213">
+        <v>100</v>
+      </c>
+      <c r="N27" s="214">
+        <v>0</v>
+      </c>
+      <c r="O27" s="214">
+        <v>93</v>
+      </c>
+      <c r="P27" s="214">
+        <v>7</v>
+      </c>
+      <c r="R27" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S27" s="216">
+        <v>0</v>
+      </c>
+      <c r="T27" s="216">
+        <v>1488000</v>
+      </c>
+      <c r="U27" s="215">
+        <v>112000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="208">
+        <v>90</v>
+      </c>
+      <c r="B28" s="209" t="s">
+        <v>295</v>
+      </c>
+      <c r="C28" s="99" t="s">
+        <v>653</v>
+      </c>
+      <c r="D28" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E28" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F28" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G28" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H28" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I28" s="212">
+        <v>41922</v>
+      </c>
+      <c r="J28" s="326">
+        <v>42287</v>
+      </c>
+      <c r="K28" s="345">
+        <v>44995</v>
+      </c>
+      <c r="L28" s="359">
+        <v>45606</v>
+      </c>
+      <c r="M28" s="213">
+        <v>90</v>
+      </c>
+      <c r="N28" s="237">
+        <v>46</v>
+      </c>
+      <c r="O28" s="214">
+        <v>44</v>
+      </c>
+      <c r="P28" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="2"/>
+      <c r="R28" s="215">
+        <v>1591800</v>
+      </c>
+      <c r="S28" s="216">
+        <v>887800</v>
+      </c>
+      <c r="T28" s="216">
+        <v>704000</v>
+      </c>
+      <c r="U28" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:22" s="79" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A29" s="155">
+        <v>91</v>
+      </c>
+      <c r="B29" s="85" t="s">
+        <v>298</v>
+      </c>
+      <c r="C29" s="98" t="s">
+        <v>654</v>
+      </c>
+      <c r="D29" s="380" t="s">
+        <v>929</v>
+      </c>
+      <c r="E29" s="97" t="s">
+        <v>18</v>
+      </c>
+      <c r="F29" s="88">
+        <v>22000</v>
+      </c>
+      <c r="G29" s="88">
+        <v>2200</v>
+      </c>
+      <c r="H29" s="88">
+        <v>19800</v>
+      </c>
+      <c r="I29" s="101">
+        <v>42109</v>
+      </c>
+      <c r="J29" s="334">
+        <v>42134</v>
+      </c>
+      <c r="K29" s="347">
+        <v>45148</v>
+      </c>
+      <c r="L29" s="361">
+        <v>45757</v>
+      </c>
+      <c r="M29" s="90">
+        <v>100</v>
+      </c>
+      <c r="N29" s="91">
+        <v>0</v>
+      </c>
+      <c r="O29" s="91">
+        <v>86</v>
+      </c>
+      <c r="P29" s="91">
+        <v>14</v>
+      </c>
+      <c r="Q29" s="100"/>
+      <c r="R29" s="92">
+        <v>2200000</v>
+      </c>
+      <c r="S29" s="93">
+        <v>0</v>
+      </c>
+      <c r="T29" s="93">
+        <v>1892000</v>
+      </c>
+      <c r="U29" s="92">
+        <v>308000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A30" s="208">
+        <v>92</v>
+      </c>
+      <c r="B30" s="226" t="s">
+        <v>302</v>
+      </c>
+      <c r="C30" s="99" t="s">
+        <v>655</v>
+      </c>
+      <c r="D30" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E30" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="211">
+        <v>22000</v>
+      </c>
+      <c r="G30" s="211">
+        <v>2200</v>
+      </c>
+      <c r="H30" s="211">
+        <v>19800</v>
+      </c>
+      <c r="I30" s="212">
+        <v>42342</v>
+      </c>
+      <c r="J30" s="326">
+        <v>42379</v>
+      </c>
+      <c r="K30" s="345">
+        <v>45392</v>
+      </c>
+      <c r="L30" s="359">
+        <v>46001</v>
+      </c>
+      <c r="M30" s="213">
+        <v>100</v>
+      </c>
+      <c r="N30" s="214">
+        <v>0</v>
+      </c>
+      <c r="O30" s="214">
+        <v>67.5</v>
+      </c>
+      <c r="P30" s="214">
+        <v>32.5</v>
+      </c>
+      <c r="Q30" s="80"/>
+      <c r="R30" s="215">
+        <v>2200000</v>
+      </c>
+      <c r="S30" s="216">
+        <v>0</v>
+      </c>
+      <c r="T30" s="216">
+        <v>1485000</v>
+      </c>
+      <c r="U30" s="215">
+        <v>715000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A31" s="155">
+        <v>94</v>
+      </c>
+      <c r="B31" s="96" t="s">
+        <v>309</v>
+      </c>
+      <c r="C31" s="99" t="s">
+        <v>657</v>
+      </c>
+      <c r="D31" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E31" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F31" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G31" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H31" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I31" s="89">
+        <v>41933</v>
+      </c>
+      <c r="J31" s="328">
+        <v>41953</v>
+      </c>
+      <c r="K31" s="347">
+        <v>44967</v>
+      </c>
+      <c r="L31" s="361">
+        <v>45575</v>
+      </c>
+      <c r="M31" s="90">
+        <v>100</v>
+      </c>
+      <c r="N31" s="95">
+        <v>55</v>
+      </c>
+      <c r="O31" s="91">
+        <v>45</v>
+      </c>
+      <c r="P31" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="80"/>
+      <c r="R31" s="92">
+        <v>1875000</v>
+      </c>
+      <c r="S31" s="93">
+        <v>1155000</v>
+      </c>
+      <c r="T31" s="93">
+        <v>720000</v>
+      </c>
+      <c r="U31" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A32" s="208">
+        <v>98</v>
+      </c>
+      <c r="B32" s="226" t="s">
+        <v>322</v>
+      </c>
+      <c r="C32" s="99" t="s">
+        <v>660</v>
+      </c>
+      <c r="D32" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E32" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F32" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G32" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H32" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I32" s="212">
+        <v>41865</v>
+      </c>
+      <c r="J32" s="326">
+        <v>41892</v>
+      </c>
+      <c r="K32" s="345">
+        <v>44905</v>
+      </c>
+      <c r="L32" s="359">
+        <v>45514</v>
+      </c>
+      <c r="M32" s="213">
+        <v>100</v>
+      </c>
+      <c r="N32" s="237">
+        <v>57</v>
+      </c>
+      <c r="O32" s="214">
+        <v>43</v>
+      </c>
+      <c r="P32" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="80"/>
+      <c r="R32" s="215">
+        <v>1714000</v>
+      </c>
+      <c r="S32" s="216">
+        <v>1026000</v>
+      </c>
+      <c r="T32" s="216">
+        <v>688000</v>
+      </c>
+      <c r="U32" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" spans="1:22" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A33" s="239">
+        <v>99</v>
+      </c>
+      <c r="B33" s="159" t="s">
+        <v>325</v>
+      </c>
+      <c r="C33" s="244" t="s">
+        <v>717</v>
+      </c>
+      <c r="D33" s="244" t="s">
+        <v>929</v>
+      </c>
+      <c r="E33" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F33" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G33" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H33" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I33" s="242">
+        <v>41928</v>
+      </c>
+      <c r="J33" s="330">
+        <v>41968</v>
+      </c>
+      <c r="K33" s="349">
+        <v>44982</v>
+      </c>
+      <c r="L33" s="349">
+        <v>45590</v>
+      </c>
+      <c r="M33" s="239">
+        <v>100</v>
+      </c>
+      <c r="N33" s="246">
+        <v>55</v>
+      </c>
+      <c r="O33" s="246">
+        <v>45</v>
+      </c>
+      <c r="P33" s="246">
+        <v>0</v>
+      </c>
+      <c r="R33" s="245">
+        <v>1710000</v>
+      </c>
+      <c r="S33" s="245">
+        <v>990000</v>
+      </c>
+      <c r="T33" s="245">
+        <v>720000</v>
+      </c>
+      <c r="U33" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A34" s="208">
+        <v>101</v>
+      </c>
+      <c r="B34" s="226" t="s">
+        <v>333</v>
+      </c>
+      <c r="C34" s="99" t="s">
+        <v>662</v>
+      </c>
+      <c r="D34" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E34" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F34" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G34" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H34" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I34" s="212">
+        <v>41804</v>
+      </c>
+      <c r="J34" s="326">
+        <v>41830</v>
+      </c>
+      <c r="K34" s="345">
+        <v>44844</v>
+      </c>
+      <c r="L34" s="359">
+        <v>45453</v>
+      </c>
+      <c r="M34" s="213">
+        <v>100</v>
+      </c>
+      <c r="N34" s="237">
+        <v>60</v>
+      </c>
+      <c r="O34" s="214">
+        <v>40</v>
+      </c>
+      <c r="P34" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="80"/>
+      <c r="R34" s="215">
+        <v>1720000</v>
+      </c>
+      <c r="S34" s="216">
+        <v>1062000</v>
+      </c>
+      <c r="T34" s="216">
+        <v>648000</v>
+      </c>
+      <c r="U34" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A35" s="155">
+        <v>104</v>
+      </c>
+      <c r="B35" s="96" t="s">
+        <v>343</v>
+      </c>
+      <c r="C35" s="99" t="s">
+        <v>664</v>
+      </c>
+      <c r="D35" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E35" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="88">
+        <v>20000</v>
+      </c>
+      <c r="G35" s="88">
+        <v>2000</v>
+      </c>
+      <c r="H35" s="88">
+        <v>18000</v>
+      </c>
+      <c r="I35" s="89">
+        <v>42111</v>
+      </c>
+      <c r="J35" s="328">
+        <v>42134</v>
+      </c>
+      <c r="K35" s="347">
+        <v>45148</v>
+      </c>
+      <c r="L35" s="361">
+        <v>45757</v>
+      </c>
+      <c r="M35" s="90">
+        <v>100</v>
+      </c>
+      <c r="N35" s="91">
+        <v>0</v>
+      </c>
+      <c r="O35" s="91">
+        <v>0</v>
+      </c>
+      <c r="P35" s="91">
+        <v>100</v>
+      </c>
+      <c r="Q35" s="2"/>
+      <c r="R35" s="92">
+        <v>2000000</v>
+      </c>
+      <c r="S35" s="93">
+        <v>0</v>
+      </c>
+      <c r="T35" s="93">
+        <v>0</v>
+      </c>
+      <c r="U35" s="92">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="36" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A36" s="155">
+        <v>105</v>
+      </c>
+      <c r="B36" s="96" t="s">
+        <v>347</v>
+      </c>
+      <c r="C36" s="99" t="s">
+        <v>665</v>
+      </c>
+      <c r="D36" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E36" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G36" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H36" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I36" s="89">
+        <v>41883</v>
+      </c>
+      <c r="J36" s="328">
+        <v>41922</v>
+      </c>
+      <c r="K36" s="347">
+        <v>44936</v>
+      </c>
+      <c r="L36" s="361">
+        <v>45545</v>
+      </c>
+      <c r="M36" s="90">
+        <v>100</v>
+      </c>
+      <c r="N36" s="95">
+        <v>56</v>
+      </c>
+      <c r="O36" s="91">
+        <v>44</v>
+      </c>
+      <c r="P36" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="80"/>
+      <c r="R36" s="92">
+        <v>2000000</v>
+      </c>
+      <c r="S36" s="93">
+        <v>1008000</v>
+      </c>
+      <c r="T36" s="93">
+        <v>992000</v>
+      </c>
+      <c r="U36" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A37" s="155">
+        <v>106</v>
+      </c>
+      <c r="B37" s="85" t="s">
+        <v>351</v>
+      </c>
+      <c r="C37" s="94" t="s">
+        <v>666</v>
+      </c>
+      <c r="D37" s="371" t="s">
+        <v>929</v>
+      </c>
+      <c r="E37" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F37" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G37" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H37" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I37" s="89">
+        <v>41711</v>
+      </c>
+      <c r="J37" s="328">
+        <v>41769</v>
+      </c>
+      <c r="K37" s="347">
+        <v>44783</v>
+      </c>
+      <c r="L37" s="361">
+        <v>45392</v>
+      </c>
+      <c r="M37" s="90">
+        <v>100</v>
+      </c>
+      <c r="N37" s="91">
+        <v>0</v>
+      </c>
+      <c r="O37" s="91">
+        <v>100</v>
+      </c>
+      <c r="P37" s="91">
+        <v>0</v>
+      </c>
+      <c r="R37" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S37" s="93">
+        <v>0</v>
+      </c>
+      <c r="T37" s="93">
+        <v>1600000</v>
+      </c>
+      <c r="U37" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A38" s="208">
+        <v>112</v>
+      </c>
+      <c r="B38" s="226" t="s">
+        <v>376</v>
+      </c>
+      <c r="C38" s="99" t="s">
+        <v>671</v>
+      </c>
+      <c r="D38" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E38" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G38" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H38" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I38" s="212">
+        <v>41814</v>
+      </c>
+      <c r="J38" s="326">
+        <v>41830</v>
+      </c>
+      <c r="K38" s="345">
+        <v>44844</v>
+      </c>
+      <c r="L38" s="359">
+        <v>45453</v>
+      </c>
+      <c r="M38" s="213">
+        <v>100</v>
+      </c>
+      <c r="N38" s="237">
+        <v>59</v>
+      </c>
+      <c r="O38" s="214">
+        <v>41</v>
+      </c>
+      <c r="P38" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q38" s="80"/>
+      <c r="R38" s="215">
+        <v>1718000</v>
+      </c>
+      <c r="S38" s="216">
+        <v>1062000</v>
+      </c>
+      <c r="T38" s="216">
+        <v>656000</v>
+      </c>
+      <c r="U38" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A39" s="208"/>
+      <c r="B39" s="226" t="s">
+        <v>381</v>
+      </c>
+      <c r="C39" s="99" t="s">
+        <v>672</v>
+      </c>
+      <c r="D39" s="373"/>
+      <c r="E39" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F39" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G39" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H39" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I39" s="212">
+        <v>41830</v>
+      </c>
+      <c r="J39" s="326">
+        <v>41861</v>
+      </c>
+      <c r="K39" s="345">
+        <v>44875</v>
+      </c>
+      <c r="L39" s="359">
+        <v>45483</v>
+      </c>
+      <c r="M39" s="213">
+        <v>100</v>
+      </c>
+      <c r="N39" s="237">
+        <v>100</v>
+      </c>
+      <c r="O39" s="214">
+        <v>0</v>
+      </c>
+      <c r="P39" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q39" s="80"/>
+      <c r="R39" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S39" s="216">
+        <v>0</v>
+      </c>
+      <c r="T39" s="216">
+        <v>0</v>
+      </c>
+      <c r="U39" s="215"/>
+    </row>
+    <row r="40" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A40" s="155">
+        <v>114</v>
+      </c>
+      <c r="B40" s="85" t="s">
+        <v>386</v>
+      </c>
+      <c r="C40" s="99" t="s">
+        <v>673</v>
+      </c>
+      <c r="D40" s="373" t="s">
+        <v>960</v>
+      </c>
+      <c r="E40" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G40" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H40" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I40" s="89">
+        <v>41890</v>
+      </c>
+      <c r="J40" s="328">
+        <v>41922</v>
+      </c>
+      <c r="K40" s="347">
+        <v>44936</v>
+      </c>
+      <c r="L40" s="361">
+        <v>45545</v>
+      </c>
+      <c r="M40" s="90">
+        <v>100</v>
+      </c>
+      <c r="N40" s="95">
+        <v>56</v>
+      </c>
+      <c r="O40" s="91">
+        <v>18</v>
+      </c>
+      <c r="P40" s="91">
+        <v>26</v>
+      </c>
+      <c r="R40" s="92">
+        <v>1712000</v>
+      </c>
+      <c r="S40" s="93">
+        <v>1008000</v>
+      </c>
+      <c r="T40" s="93">
+        <v>288000</v>
+      </c>
+      <c r="U40" s="92">
+        <v>416000</v>
+      </c>
+      <c r="V40" s="80" t="s">
+        <v>959</v>
+      </c>
+    </row>
+    <row r="41" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A41" s="239">
+        <v>115</v>
+      </c>
+      <c r="B41" s="159" t="s">
+        <v>389</v>
+      </c>
+      <c r="C41" s="240" t="s">
+        <v>674</v>
+      </c>
+      <c r="D41" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E41" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F41" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G41" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H41" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I41" s="242">
+        <v>41926</v>
+      </c>
+      <c r="J41" s="330">
+        <v>41998</v>
+      </c>
+      <c r="K41" s="349">
+        <v>45010</v>
+      </c>
+      <c r="L41" s="349">
+        <v>45621</v>
+      </c>
+      <c r="M41" s="239">
+        <v>100</v>
+      </c>
+      <c r="N41" s="246">
+        <v>54</v>
+      </c>
+      <c r="O41" s="246">
+        <v>46</v>
+      </c>
+      <c r="P41" s="246">
+        <v>0</v>
+      </c>
+      <c r="R41" s="245">
+        <v>1708000</v>
+      </c>
+      <c r="S41" s="245">
+        <v>972000</v>
+      </c>
+      <c r="T41" s="245">
+        <v>736000</v>
+      </c>
+      <c r="U41" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A42" s="239"/>
+      <c r="B42" s="159" t="s">
+        <v>397</v>
+      </c>
+      <c r="C42" s="240" t="s">
+        <v>676</v>
+      </c>
+      <c r="D42" s="240"/>
+      <c r="E42" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F42" s="241">
+        <v>22000</v>
+      </c>
+      <c r="G42" s="241">
+        <v>2200</v>
+      </c>
+      <c r="H42" s="241">
+        <v>19800</v>
+      </c>
+      <c r="I42" s="242">
+        <v>42149</v>
+      </c>
+      <c r="J42" s="330">
+        <v>42180</v>
+      </c>
+      <c r="K42" s="349">
+        <v>45194</v>
+      </c>
+      <c r="L42" s="349">
+        <v>45802</v>
+      </c>
+      <c r="M42" s="239">
+        <v>100</v>
+      </c>
+      <c r="N42" s="246">
+        <v>0</v>
+      </c>
+      <c r="O42" s="246">
+        <v>100</v>
+      </c>
+      <c r="P42" s="246">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="80"/>
+      <c r="R42" s="245">
+        <v>2200000</v>
+      </c>
+      <c r="S42" s="245">
+        <v>0</v>
+      </c>
+      <c r="T42" s="245">
+        <v>2200000</v>
+      </c>
+      <c r="U42" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:22" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A43" s="239">
+        <v>119</v>
+      </c>
+      <c r="B43" s="159" t="s">
+        <v>406</v>
+      </c>
+      <c r="C43" s="240" t="s">
+        <v>678</v>
+      </c>
+      <c r="D43" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E43" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F43" s="241">
+        <v>22000</v>
+      </c>
+      <c r="G43" s="241">
+        <v>2200</v>
+      </c>
+      <c r="H43" s="241">
+        <v>19800</v>
+      </c>
+      <c r="I43" s="242">
+        <v>42356</v>
+      </c>
+      <c r="J43" s="330">
+        <v>42394</v>
+      </c>
+      <c r="K43" s="349">
+        <v>45407</v>
+      </c>
+      <c r="L43" s="349">
+        <v>46016</v>
+      </c>
+      <c r="M43" s="239">
+        <v>100</v>
+      </c>
+      <c r="N43" s="246">
+        <v>0</v>
+      </c>
+      <c r="O43" s="246">
+        <v>95</v>
+      </c>
+      <c r="P43" s="246">
+        <v>5</v>
+      </c>
+      <c r="Q43" s="80"/>
+      <c r="R43" s="245">
+        <v>2200000</v>
+      </c>
+      <c r="S43" s="245">
+        <v>0</v>
+      </c>
+      <c r="T43" s="245">
+        <v>2090000</v>
+      </c>
+      <c r="U43" s="245">
+        <v>110000</v>
+      </c>
+    </row>
+    <row r="44" spans="1:22" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A44" s="239">
+        <v>125</v>
+      </c>
+      <c r="B44" s="159" t="s">
+        <v>434</v>
+      </c>
+      <c r="C44" s="240" t="s">
+        <v>683</v>
+      </c>
+      <c r="D44" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E44" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F44" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G44" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H44" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I44" s="242">
+        <v>41912</v>
+      </c>
+      <c r="J44" s="330">
+        <v>41937</v>
+      </c>
+      <c r="K44" s="349">
+        <v>44951</v>
+      </c>
+      <c r="L44" s="349">
+        <v>45560</v>
+      </c>
+      <c r="M44" s="239">
+        <v>100</v>
+      </c>
+      <c r="N44" s="246">
+        <v>45</v>
+      </c>
+      <c r="O44" s="246">
+        <v>55</v>
+      </c>
+      <c r="P44" s="246">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="80"/>
+      <c r="R44" s="245">
+        <v>1690000</v>
+      </c>
+      <c r="S44" s="245">
+        <v>810000</v>
+      </c>
+      <c r="T44" s="245">
+        <v>816000</v>
+      </c>
+      <c r="U44" s="245" t="s">
+        <v>790</v>
+      </c>
+    </row>
+    <row r="45" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A45" s="208">
+        <v>126</v>
+      </c>
+      <c r="B45" s="226" t="s">
+        <v>437</v>
+      </c>
+      <c r="C45" s="99" t="s">
+        <v>684</v>
+      </c>
+      <c r="D45" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E45" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F45" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G45" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H45" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I45" s="212">
+        <v>41900</v>
+      </c>
+      <c r="J45" s="326">
+        <v>41922</v>
+      </c>
+      <c r="K45" s="345">
+        <v>44936</v>
+      </c>
+      <c r="L45" s="359">
+        <v>45545</v>
+      </c>
+      <c r="M45" s="213">
+        <v>100</v>
+      </c>
+      <c r="N45" s="237">
+        <v>58</v>
+      </c>
+      <c r="O45" s="214">
+        <v>42</v>
+      </c>
+      <c r="P45" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="80"/>
+      <c r="R45" s="215">
+        <v>1716000</v>
+      </c>
+      <c r="S45" s="216">
+        <v>1044000</v>
+      </c>
+      <c r="T45" s="216">
+        <v>672000</v>
+      </c>
+      <c r="U45" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:22" s="78" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A46" s="394">
+        <v>133</v>
+      </c>
+      <c r="B46" s="159" t="s">
+        <v>467</v>
+      </c>
+      <c r="C46" s="240" t="s">
+        <v>688</v>
+      </c>
+      <c r="D46" s="240" t="s">
+        <v>929</v>
+      </c>
+      <c r="E46" s="241" t="s">
+        <v>30</v>
+      </c>
+      <c r="F46" s="241">
+        <v>16000</v>
+      </c>
+      <c r="G46" s="241">
+        <v>1600</v>
+      </c>
+      <c r="H46" s="241">
+        <v>14400</v>
+      </c>
+      <c r="I46" s="242">
+        <v>41819</v>
+      </c>
+      <c r="J46" s="330">
+        <v>41876</v>
+      </c>
+      <c r="K46" s="349">
+        <v>44890</v>
+      </c>
+      <c r="L46" s="349">
+        <v>45498</v>
+      </c>
+      <c r="M46" s="239">
+        <v>100</v>
+      </c>
+      <c r="N46" s="246">
+        <v>61</v>
+      </c>
+      <c r="O46" s="246">
+        <v>39</v>
+      </c>
+      <c r="P46" s="246">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="80"/>
+      <c r="R46" s="245">
+        <v>1722000</v>
+      </c>
+      <c r="S46" s="245">
+        <v>1098000</v>
+      </c>
+      <c r="T46" s="245">
+        <v>624000</v>
+      </c>
+      <c r="U46" s="245">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:22" s="80" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A47" s="155">
+        <v>134</v>
+      </c>
+      <c r="B47" s="85" t="s">
+        <v>472</v>
+      </c>
+      <c r="C47" s="99" t="s">
+        <v>689</v>
+      </c>
+      <c r="D47" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E47" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F47" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G47" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H47" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I47" s="89">
+        <v>41711</v>
+      </c>
+      <c r="J47" s="328">
+        <v>41769</v>
+      </c>
+      <c r="K47" s="347">
+        <v>44783</v>
+      </c>
+      <c r="L47" s="361">
+        <v>45392</v>
+      </c>
+      <c r="M47" s="90">
+        <v>100</v>
+      </c>
+      <c r="N47" s="91">
+        <v>0</v>
+      </c>
+      <c r="O47" s="91">
+        <v>100</v>
+      </c>
+      <c r="P47" s="91">
+        <v>0</v>
+      </c>
+      <c r="R47" s="92">
+        <v>1600000</v>
+      </c>
+      <c r="S47" s="93">
+        <v>0</v>
+      </c>
+      <c r="T47" s="93">
+        <v>1600000</v>
+      </c>
+      <c r="U47" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:22" s="78" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A48" s="155">
+        <v>139</v>
+      </c>
+      <c r="B48" s="96" t="s">
+        <v>494</v>
+      </c>
+      <c r="C48" s="94" t="s">
+        <v>694</v>
+      </c>
+      <c r="D48" s="371" t="s">
+        <v>929</v>
+      </c>
+      <c r="E48" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F48" s="88">
+        <v>16000</v>
+      </c>
+      <c r="G48" s="88">
+        <v>1600</v>
+      </c>
+      <c r="H48" s="88">
+        <v>14400</v>
+      </c>
+      <c r="I48" s="89">
+        <v>41827</v>
+      </c>
+      <c r="J48" s="328">
+        <v>41861</v>
+      </c>
+      <c r="K48" s="347">
+        <v>44875</v>
+      </c>
+      <c r="L48" s="361">
+        <v>45483</v>
+      </c>
+      <c r="M48" s="90">
+        <v>100</v>
+      </c>
+      <c r="N48" s="95">
+        <v>58</v>
+      </c>
+      <c r="O48" s="91">
+        <v>42</v>
+      </c>
+      <c r="P48" s="91">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="80"/>
+      <c r="R48" s="92">
+        <v>1716000</v>
+      </c>
+      <c r="S48" s="93">
+        <v>1044000</v>
+      </c>
+      <c r="T48" s="93">
+        <v>672000</v>
+      </c>
+      <c r="U48" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:21" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A49" s="208">
+        <v>143</v>
+      </c>
+      <c r="B49" s="226" t="s">
+        <v>499</v>
+      </c>
+      <c r="C49" s="99" t="s">
+        <v>696</v>
+      </c>
+      <c r="D49" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E49" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F49" s="211">
+        <v>16000</v>
+      </c>
+      <c r="G49" s="211">
+        <v>1600</v>
+      </c>
+      <c r="H49" s="211">
+        <v>14400</v>
+      </c>
+      <c r="I49" s="212">
+        <v>41586</v>
+      </c>
+      <c r="J49" s="326">
+        <v>41618</v>
+      </c>
+      <c r="K49" s="345">
+        <v>44630</v>
+      </c>
+      <c r="L49" s="359">
+        <v>45240</v>
+      </c>
+      <c r="M49" s="213">
+        <v>100</v>
+      </c>
+      <c r="N49" s="214">
+        <v>0</v>
+      </c>
+      <c r="O49" s="214">
+        <v>100</v>
+      </c>
+      <c r="P49" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="80"/>
+      <c r="R49" s="215">
+        <v>1600000</v>
+      </c>
+      <c r="S49" s="216">
+        <v>0</v>
+      </c>
+      <c r="T49" s="216">
+        <v>1600000</v>
+      </c>
+      <c r="U49" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:21" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A50" s="155">
+        <v>146</v>
+      </c>
+      <c r="B50" s="96" t="s">
+        <v>510</v>
+      </c>
+      <c r="C50" s="94" t="s">
+        <v>698</v>
+      </c>
+      <c r="D50" s="371" t="s">
+        <v>929</v>
+      </c>
+      <c r="E50" s="87" t="s">
+        <v>18</v>
+      </c>
+      <c r="F50" s="88">
+        <v>22000</v>
+      </c>
+      <c r="G50" s="88">
+        <v>2200</v>
+      </c>
+      <c r="H50" s="88">
+        <v>19800</v>
+      </c>
+      <c r="I50" s="89">
+        <v>42084</v>
+      </c>
+      <c r="J50" s="328">
+        <v>42104</v>
+      </c>
+      <c r="K50" s="347">
+        <v>45117</v>
+      </c>
+      <c r="L50" s="361">
+        <v>45726</v>
+      </c>
+      <c r="M50" s="90">
+        <v>100</v>
+      </c>
+      <c r="N50" s="91">
+        <v>0</v>
+      </c>
+      <c r="O50" s="91">
+        <v>100</v>
+      </c>
+      <c r="P50" s="91">
+        <v>0</v>
+      </c>
+      <c r="R50" s="92">
+        <v>2200000</v>
+      </c>
+      <c r="S50" s="93">
+        <v>0</v>
+      </c>
+      <c r="T50" s="93">
+        <v>2200000</v>
+      </c>
+      <c r="U50" s="92">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:21" s="2" customFormat="1" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="208">
+        <v>148</v>
+      </c>
+      <c r="B51" s="226" t="s">
+        <v>517</v>
+      </c>
+      <c r="C51" s="99" t="s">
+        <v>699</v>
+      </c>
+      <c r="D51" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E51" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F51" s="211">
+        <v>22000</v>
+      </c>
+      <c r="G51" s="211">
+        <v>2200</v>
+      </c>
+      <c r="H51" s="211">
+        <v>19800</v>
+      </c>
+      <c r="I51" s="212">
+        <v>42289</v>
+      </c>
+      <c r="J51" s="326">
+        <v>42318</v>
+      </c>
+      <c r="K51" s="345">
+        <v>45332</v>
+      </c>
+      <c r="L51" s="359">
+        <v>45940</v>
+      </c>
+      <c r="M51" s="213">
+        <v>100</v>
+      </c>
+      <c r="N51" s="214">
+        <v>0</v>
+      </c>
+      <c r="O51" s="214">
+        <v>100</v>
+      </c>
+      <c r="P51" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="80"/>
+      <c r="R51" s="215">
+        <v>2200000</v>
+      </c>
+      <c r="S51" s="216">
+        <v>0</v>
+      </c>
+      <c r="T51" s="216">
+        <v>2200000</v>
+      </c>
+      <c r="U51" s="215">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:21" s="2" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A52" s="208">
+        <v>149</v>
+      </c>
+      <c r="B52" s="226" t="s">
+        <v>522</v>
+      </c>
+      <c r="C52" s="99" t="s">
+        <v>699</v>
+      </c>
+      <c r="D52" s="373" t="s">
+        <v>929</v>
+      </c>
+      <c r="E52" s="210" t="s">
+        <v>18</v>
+      </c>
+      <c r="F52" s="211">
+        <v>22000</v>
+      </c>
+      <c r="G52" s="211">
+        <v>2200</v>
+      </c>
+      <c r="H52" s="211">
+        <v>19800</v>
+      </c>
+      <c r="I52" s="212">
+        <v>42289</v>
+      </c>
+      <c r="J52" s="326">
+        <v>42318</v>
+      </c>
+      <c r="K52" s="345">
+        <v>45332</v>
+      </c>
+      <c r="L52" s="359">
+        <v>45940</v>
+      </c>
+      <c r="M52" s="213">
+        <v>100</v>
+      </c>
+      <c r="N52" s="214">
+        <v>0</v>
+      </c>
+      <c r="O52" s="214">
+        <v>100</v>
+      </c>
+      <c r="P52" s="214">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="80"/>
+      <c r="R52" s="215">
+        <v>2200000</v>
+      </c>
+      <c r="S52" s="216">
+        <v>0</v>
+      </c>
+      <c r="T52" s="216">
+        <v>2200000</v>
+      </c>
+      <c r="U52" s="215">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:T41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>